<commit_message>
Panele: regeneracja z JSON (Kopalnia miedzi, prog wzrostu 2x) — sync JSON->Excel
Panel-A..E odswiezone gen-panel-*.py z aktualnych gra/data. Round-trip B/C/D OK.
Znane luki (do pozniej): (1) gen-panel-a.py hardcoduje METAL_DEPOSIT_MIN_ERA={miedz,zelazo} -> wegiel:8
z map-gen-params.json nie trafia do arkusza (wegiel i tak odlozony); (2) test roundtrip A FAIL na
legacy arkuszu Plony-terenow (pre-existing niespojnosc gen-panel-a vs export-a, niezwiazane z ta zmiana).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/panele-sterowania/Panel-A.xlsx
+++ b/panele-sterowania/Panel-A.xlsx
@@ -3981,12 +3981,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>popalnia_brazu.koszt_praca</t>
+          <t>kopalnia_miedzi.koszt_praca</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Popalnia brązu — Koszt budowy</t>
+          <t>Kopalnia miedzi — Koszt budowy</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>ulepszenie popalnia_brazu · placement/render MAPA</t>
+          <t>ulepszenie kopalnia_miedzi · placement/render MAPA</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4017,12 +4017,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>popalnia_brazu.epoka</t>
+          <t>kopalnia_miedzi.epoka</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Popalnia brązu — Epoka odblokowania</t>
+          <t>Kopalnia miedzi — Epoka odblokowania</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>ulepszenie popalnia_brazu · placement/render MAPA</t>
+          <t>ulepszenie kopalnia_miedzi · placement/render MAPA</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4053,12 +4053,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>popalnia_brazu.surowiecOdblokowany</t>
+          <t>kopalnia_miedzi.surowiecOdblokowany</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Popalnia brązu — Odblokowany surowiec (ASCII)</t>
+          <t>Kopalnia miedzi — Odblokowany surowiec (ASCII)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>ulepszenie popalnia_brazu · placement/render MAPA</t>
+          <t>ulepszenie kopalnia_miedzi · placement/render MAPA</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4091,12 +4091,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>popalnia_brazu.bonus.praca</t>
+          <t>kopalnia_miedzi.bonus.praca</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Popalnia brązu — bonus praca</t>
+          <t>Kopalnia miedzi — bonus praca</t>
         </is>
       </c>
       <c r="D46" t="n">

</xml_diff>

<commit_message>
chore(civ): sync paneli Excel A-E z JSON + fix gen-panel-d (tablica tokenow)
Panele sterowania (JSON->Excel, kierunek jednostronny) dociagniete do biezacego
gra/data. JSON gry NIETKNIETY (weryfikowane git status po kazdym generatorze).

- Panel-A/B/C/D/E zregenerowane z aktualnego JSON (gen-panel-{a..e}.py).
  Panel-C (jednostki: typy EN, Slinger, Surowiec zelazo, usuniete Legion/Kusznik)
  + Panel-D (cywilizacje: naprawione tokeny jednostek specjalnych).
- Fix gen-panel-d.py: jednostka_specjalna.wartosc jest teraz tablica (string[]);
  laczymy tokeny "/" do komorki (openpyxl nie wpisze listy).
- Round-trip test-panel-{b,c,d}-roundtrip = OK. Panel-A fail (Plony-terenow) =
  PRE-ISTNIEJACY (deprecated arkusz, potwierdzone na starym pliku), nie regresja.
- STAN-PRACY-HANDOFF.md: zaktualizowany o deploy a44d5350 (zelazo + panele).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/panele-sterowania/Panel-A.xlsx
+++ b/panele-sterowania/Panel-A.xlsx
@@ -596,7 +596,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>gen-panel-a.py · 2026-07-09</t>
+          <t>gen-panel-a.py · 2026-07-19</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">

</xml_diff>

<commit_message>
sync(panele): regeneracja Panel-A/B/C z JSON (JSON->Excel); log luki generatora kosztow surowcowych
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fs7eokPtaxbQL7KGTXXeWS
</commit_message>
<xml_diff>
--- a/panele-sterowania/Panel-A.xlsx
+++ b/panele-sterowania/Panel-A.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_INFO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ulepszenia-FOOD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ulepszenia-inne" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plony-terenow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ruch-po-terenie" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zasięgi-mgła" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generator-rozmiary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zloza-generator" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generator-E2" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa-skala" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Eksporty" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="_INFO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ulepszenia-FOOD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ulepszenia-inne" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Plony-terenow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ruch-po-terenie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Zasięgi-mgła" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Generator-rozmiary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Zloza-generator" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Generator-E2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Mapa-skala" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="_Eksporty" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -596,7 +596,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>gen-panel-a.py · 2026-07-19</t>
+          <t>gen-panel-a.py · 2026-07-24</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -7771,7 +7771,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -7811,7 +7811,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>